<commit_message>
fix: captura e unifica nome e sobrenome na extracao de pdf e cadastro do portal fake
</commit_message>
<xml_diff>
--- a/HyperAutomation/resources/Status_SAC.xlsx
+++ b/HyperAutomation/resources/Status_SAC.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,17 +40,11 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00166534"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00991B1B"/>
+      <color rgb="0092400E"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -64,12 +58,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -99,14 +88,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -548,12 +536,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>#SAC-2026-3135</t>
+          <t>#SAC-2026-1653</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>23/08/2026 22:11:27</t>
+          <t>24/08/2026 11:01:59</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -578,39 +566,39 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>SUCESSO</t>
+          <t>DUPLICADO</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>CONFIRMACAO_ENVIADA</t>
+          <t>NOTIFICACAO_ERRO_ENVIADA</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Cadastro realizado com sucesso</t>
+          <t>Cadastro duplicado: CPF já existente na base de dados do Portal Fake</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Enviado com sucesso</t>
+          <t>Não enviado (Opção desativada)</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>23/08/2026 22:11:31</t>
+          <t>24/08/2026 11:01:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>#SAC-2026-8809</t>
+          <t>#SAC-2026-4292</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>23/08/2026 22:11:27</t>
+          <t>24/08/2026 11:01:59</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -635,44 +623,44 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>SUCESSO</t>
+          <t>DUPLICADO</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>CONFIRMACAO_ENVIADA</t>
+          <t>NOTIFICACAO_ERRO_ENVIADA</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Cadastro realizado com sucesso</t>
+          <t>Cadastro duplicado: CPF já existente na base de dados do Portal Fake</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Enviado com sucesso</t>
+          <t>Não enviado (Opção desativada)</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>23/08/2026 22:11:35</t>
+          <t>24/08/2026 11:01:59</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>#SAC-2026-8816</t>
+          <t>#SAC-2026-2122</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>23/08/2026 22:11:27</t>
+          <t>24/08/2026 11:01:59</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Fani</t>
+          <t>Fani Batista</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -692,39 +680,39 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>ERRO_CADASTRO</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
+          <t>DUPLICADO</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>NOTIFICACAO_ERRO_ENVIADA</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Erro no preenchimento/validação do formulário: Erro na validação do formulário</t>
+          <t>Cadastro duplicado: CPF já existente na base de dados do Portal Fake</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Enviado com sucesso</t>
+          <t>Não enviado (Opção desativada)</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>23/08/2026 22:11:38</t>
+          <t>24/08/2026 11:01:59</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>#SAC-2026-5467</t>
+          <t>#SAC-2026-6072</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>23/08/2026 22:11:27</t>
+          <t>24/08/2026 11:01:59</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -749,27 +737,27 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>SUCESSO</t>
+          <t>DUPLICADO</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>CONFIRMACAO_ENVIADA</t>
+          <t>NOTIFICACAO_ERRO_ENVIADA</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Cadastro realizado com sucesso</t>
+          <t>Cadastro duplicado: CPF já existente na base de dados do Portal Fake</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Enviado com sucesso</t>
+          <t>Não enviado (Opção desativada)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>23/08/2026 22:11:42</t>
+          <t>24/08/2026 11:01:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug do processo 1 e 2 resolvido
</commit_message>
<xml_diff>
--- a/HyperAutomation/resources/Status_SAC.xlsx
+++ b/HyperAutomation/resources/Status_SAC.xlsx
@@ -536,32 +536,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>#SAC-2026-7378</t>
+          <t>#SAC-2026-8414</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>24/08/2026 17:41:46</t>
+          <t>24/08/2026 22:16:22</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Sannyer Nery</t>
+          <t>Fani Batista</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>035.360.542-50</t>
+          <t>02033414221</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>portalfakeifam@gmail.com</t>
+          <t>fani.souza19@gmail.com</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>(92) 99982-7524</t>
+          <t>(92) 99503-7524</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>24/08/2026 17:41:52</t>
+          <t>24/08/2026 22:16:25</t>
         </is>
       </c>
     </row>

</xml_diff>